<commit_message>
backup before exotel api changes
</commit_message>
<xml_diff>
--- a/campaigns.xlsx
+++ b/campaigns.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="45">
   <si>
     <t>organization_name</t>
   </si>
@@ -58,7 +58,7 @@
     <t>Delhi</t>
   </si>
   <si>
-    <t>+919876543210</t>
+    <t>09816463933</t>
   </si>
   <si>
     <t>Sunrise Finance</t>
@@ -82,9 +82,6 @@
     <t>Mumbai</t>
   </si>
   <si>
-    <t>+919812345678</t>
-  </si>
-  <si>
     <t>GreenLeaf Realty</t>
   </si>
   <si>
@@ -104,9 +101,6 @@
   </si>
   <si>
     <t>Pune</t>
-  </si>
-  <si>
-    <t>+919900112233</t>
   </si>
   <si>
     <t>GoodHealth Clinic</t>
@@ -178,12 +172,18 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="9"/>
+        <bgColor auto="1"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -196,16 +196,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </left>
       <right style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </right>
       <top style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="9"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -222,10 +222,10 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -245,6 +245,7 @@
       <rgbColor rgb="ffff00ff"/>
       <rgbColor rgb="ff00ffff"/>
       <rgbColor rgb="ff000000"/>
+      <rgbColor rgb="ffffffff"/>
       <rgbColor rgb="ffaaaaaa"/>
     </indexedColors>
   </colors>
@@ -396,9 +397,9 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -478,7 +479,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -505,10 +506,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -755,9 +756,9 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
             <a:srgbClr val="000000">
-              <a:alpha val="38000"/>
+              <a:alpha val="35000"/>
             </a:srgbClr>
           </a:outerShdw>
         </a:effectLst>
@@ -1035,7 +1036,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1062,10 +1063,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1396,38 +1397,38 @@
         <v>22</v>
       </c>
       <c r="H3" t="s" s="2">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" ht="13.55" customHeight="1">
       <c r="A4" t="s" s="2">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s" s="2">
         <v>24</v>
       </c>
-      <c r="B4" t="s" s="2">
+      <c r="C4" t="s" s="2">
         <v>25</v>
       </c>
-      <c r="C4" t="s" s="2">
+      <c r="D4" t="s" s="2">
         <v>26</v>
       </c>
-      <c r="D4" t="s" s="2">
+      <c r="E4" t="s" s="2">
         <v>27</v>
       </c>
-      <c r="E4" t="s" s="2">
+      <c r="F4" t="s" s="2">
         <v>28</v>
       </c>
-      <c r="F4" t="s" s="2">
+      <c r="G4" t="s" s="2">
         <v>29</v>
       </c>
-      <c r="G4" t="s" s="2">
-        <v>30</v>
-      </c>
       <c r="H4" t="s" s="2">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="13.55" customHeight="1">
       <c r="A5" t="s" s="2">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s" s="2">
         <v>9</v>
@@ -1436,16 +1437,16 @@
         <v>10</v>
       </c>
       <c r="D5" t="s" s="2">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="F5" t="s" s="2">
         <v>33</v>
       </c>
-      <c r="E5" t="s" s="2">
+      <c r="G5" t="s" s="2">
         <v>34</v>
-      </c>
-      <c r="F5" t="s" s="2">
-        <v>35</v>
-      </c>
-      <c r="G5" t="s" s="2">
-        <v>36</v>
       </c>
       <c r="H5" t="s" s="2">
         <v>15</v>
@@ -1453,7 +1454,7 @@
     </row>
     <row r="6" ht="13.55" customHeight="1">
       <c r="A6" t="s" s="2">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s" s="2">
         <v>17</v>
@@ -1462,45 +1463,45 @@
         <v>18</v>
       </c>
       <c r="D6" t="s" s="2">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s" s="2">
+        <v>37</v>
+      </c>
+      <c r="F6" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="E6" t="s" s="2">
+      <c r="G6" t="s" s="2">
         <v>39</v>
       </c>
-      <c r="F6" t="s" s="2">
-        <v>40</v>
-      </c>
-      <c r="G6" t="s" s="2">
-        <v>41</v>
-      </c>
       <c r="H6" t="s" s="2">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="13.55" customHeight="1">
       <c r="A7" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s" s="2">
         <v>42</v>
       </c>
-      <c r="B7" t="s" s="2">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s" s="2">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s" s="2">
+      <c r="F7" t="s" s="2">
         <v>43</v>
       </c>
-      <c r="E7" t="s" s="2">
+      <c r="G7" t="s" s="2">
         <v>44</v>
       </c>
-      <c r="F7" t="s" s="2">
-        <v>45</v>
-      </c>
-      <c r="G7" t="s" s="2">
-        <v>46</v>
-      </c>
       <c r="H7" t="s" s="2">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" ht="13.55" customHeight="1">

</xml_diff>